<commit_message>
Recopied in the CF_ input xlsx files as I thought they might have had an error.
</commit_message>
<xml_diff>
--- a/Inputs/CF_template_parameters_Exposure.xlsx
+++ b/Inputs/CF_template_parameters_Exposure.xlsx
@@ -3456,6 +3456,13 @@
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="41d9f072-86bf-4c63-b117-debf50ff4701">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
   </documentManagement>
 </p:properties>
 </file>
@@ -3964,5 +3971,5 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3ED7FF5-C43E-4D13-A7AA-85AF391460D9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74E43103-4BB8-4F2E-AC53-ED5EAA6897C8}"/>
 </file>
</xml_diff>